<commit_message>
Add newsletter signup block to Stay Up to Date section
The "Stay Up to Date with Compliance" section rendered with only the heading +
copy — no email input/button. The source form is a dynamic HubSpot embed absent
from static HTML, and the section had been mapped to the heavyweight Adaptive
Form 'form' block for which no parser ran, so nothing rendered.

Add a lightweight 'newsletter' block: email input + orange Sign Up button
(demo submit shows a thank-you), styled to match the live dark section. Wire
rc9 to it: newsletter parser emits the block + preserves the heading/copy;
block registered in the Universal Editor (section filter + xwalk model with
placeholder/cta/action fields). Field-hinted single-column rows so it also
round-trips into the JCR package; block reads them positionally at runtime.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["cards-promo","cards-category","cards-product","tabs-industry","cards-review","cards-blog","cards-value"]</t>
+    <t>["cards-promo","cards-category","cards-product","tabs-industry","cards-review","cards-blog","cards-value","newsletter"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-24T14:47:21.561Z</t>
+    <t>2026-09-24T15:17:30.773Z</t>
   </si>
   <si>
     <t>Safety Signs, Tags, Labels - Guaranteed Compliance</t>

</xml_diff>